<commit_message>
auto: cambios de la sesion de Claude en claude/calcularya-paridad
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 8/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 9/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 8/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 9/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
auto: cambios de la sesion de Claude en claude/program-audit-production-e5007a
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 9/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 13/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 9/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 13/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
datos-vivos: ipc, plazofijo, canasta-crianza (2026-10-14)
- Serie del IPC (INDEC vía datos.gob.ar): fecha de consulta refrescada (la guardada era del 2026-10-07)
- TNA (BCRA) e inflación de referencia de /plazo-fijo: 🔄 TNA_FALLBACK 22.3% (2026-10-08) → 20.65% (2026-10-13) · BCRA serie 12. | ✓ INFLACION_DEFAULT al día (1.7% · agosto 2026).
- Canasta de crianza (INDEC): fecha de consulta refrescada (la guardada era del 2026-10-07)

Commit automático del workflow datos-vivos: cada dato pasó sus checks y check-all completo.
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 9/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 14/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 9/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 14/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46304</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
datos-vivos: plazofijo, canasta-basica, jubilaciones (2026-10-15)
- TNA (BCRA) e inflación de referencia de /plazo-fijo: 🔄 TNA_FALLBACK 20.65% (2026-10-13) → 20.85% (2026-10-14) · BCRA serie 12. | ✓ INFLACION_DEFAULT al día (1.7% · agosto 2026).
- Canasta básica CBA/CBT (INDEC): fecha de consulta refrescada (la guardada era del 2026-10-07)
- Serie del haber mínimo (ANSES vía datos.gob.ar): fecha de consulta refrescada (la guardada era del 2026-10-07)

Commit automático del workflow datos-vivos: cada dato pasó sus checks y check-all completo.
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 14/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 15/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 14/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 15/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
datos-vivos: plazofijo, uma (2026-10-19)
- TNA (BCRA) e inflación de referencia de /plazo-fijo: 🔄 TNA_FALLBACK 21.74% (2026-10-15) → 22.66% (2026-10-16) · BCRA serie 12. | ✓ INFLACION_DEFAULT al día (1.7% · agosto 2026).
- UMA de honorarios (resoluciones de la CSJN): ⚠️  22 resolución(es) vienen escaneadas (PDF sin texto) y quedan fuera de la serie: 936 (22/05/2025), 580 (25/04/2025), 237 (18/03/2025), 3495 (19/12/2024), 2910 (07/11/2024), 2375 (12/09/2024), 1497 (06/06/2024), 925 (30/04/2024), 626 (04/04/2024), 176 (21/02/2024), 2722 (12/10/2023), 9/2023 (04/04/2023), 12/2022 (23/05/2022), 4/2022 (11/03/2022), 21/2021 (01/10/2021), 12/2021 (13/07/2021), 7/2021 (20/04/2021), 1/2021 (23/02/2021), 36/2020 (30/11/2020), 30/2019 (21/11/2019), 20/2019 (16/07/2019), 13/2018 (03/05/2018) | 🔄 UMA nueva: $105.991 desde 2026-08-01 (Res. SGA 2372/2026)

Novedades:
- uma-2026-08 · UMA de agosto: $ 105.991

Commit automático del workflow datos-vivos: cada dato pasó sus checks y check-all completo.
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 16/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 19/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 16/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 19/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
planillas: desplegables que leen su misma hoja (Comercio y calcularya) + check para todas
Comercio (Liquidación!B5) y 7 planillas de calcularya (cl, do, ec, mx, ni, pe, sv) tenían
desplegables que leían 'Escala 2026' o 'Tablas oficiales': en Google Sheets salen vacíos o corridos.
Ahora cada uno lee una columna oculta de su hoja y lleva su propio mensaje de error.
check_planillas_desplegables recorre todos los .xlsx de private/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 19/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 20/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 19/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 20/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
planillas: desplegables que leen su misma hoja (Comercio y calcularya) + check para todas (#55)
Comercio (Liquidación!B5) y 7 planillas de calcularya (cl, do, ec, mx, ni, pe, sv) tenían
desplegables que leían 'Escala 2026' o 'Tablas oficiales': en Google Sheets salen vacíos o corridos.
Ahora cada uno lee una columna oculta de su hoja y lleva su propio mensaje de error.
check_planillas_desplegables recorre todos los .xlsx de private/.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 19/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 20/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 19/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 20/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
datos-vivos: ipc, canasta-basica, jubilaciones (2026-10-22)
- Serie del IPC (INDEC vía datos.gob.ar): fecha de consulta refrescada (la guardada era del 2026-10-15)
- Canasta básica CBA/CBT (INDEC): fecha de consulta refrescada (la guardada era del 2026-10-15)
- Serie del haber mínimo (ANSES vía datos.gob.ar): fecha de consulta refrescada (la guardada era del 2026-10-15)

Commit automático del workflow datos-vivos: cada dato pasó sus checks y check-all completo.
</commit_message>
<xml_diff>
--- a/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/bo/sueldo-y-liquidacion-2026.xlsx
@@ -32,7 +32,7 @@
     <t>«Finiquito»: pone sus fechas, su promedio y cómo terminó el trabajo, y le dice la indemnización, el desahucio, el aguinaldo y las vacaciones.</t>
   </si>
   <si>
-    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 21/10/2026.</t>
+    <t>«Tablas oficiales» tiene cada valor oficial que usan las fórmulas, con el enlace a su fuente y la fecha en que lo verificamos. Los valores son los vigentes al 22/10/2026.</t>
   </si>
   <si>
     <t>Cuando cambia un valor oficial, actualizamos la planilla y el mismo enlace de descarga le baja la versión nueva.</t>
@@ -266,7 +266,7 @@
     <t>Tablas oficiales de Bolivia</t>
   </si>
   <si>
-    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 21/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
+    <t>Son los valores que usan las fórmulas de esta planilla, vigentes al 22/10/2026. Cada uno trae el enlace a la norma o al organismo que lo publica y la fecha en que lo verificamos.</t>
   </si>
   <si>
     <t>Dato</t>
@@ -1615,7 +1615,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="20">
-        <v>46316</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>